<commit_message>
Fixed missing depth for a handful of 2016 sites and one SuRGE site. Fixed inspectMeasurementValues.R. Updated data_paper files.
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/beaulieu_jake_epa_gov/Documents/gitRepository/SuRGE/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30E28EBA-695B-4B28-8321-9B2E01519D99}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5BB1541-24BC-4185-B360-2E8261798A7C}"/>
   <bookViews>
-    <workbookView xWindow="4488" yWindow="5112" windowWidth="40200" windowHeight="12516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="18576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1312,6 +1312,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -2637,6 +2641,9 @@
       <c r="L10" t="s">
         <v>198</v>
       </c>
+      <c r="W10">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="11" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
@@ -4357,8 +4364,45 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4833,45 +4877,8 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4883,9 +4890,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4914,15 +4927,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added missing depth to 70_riverine data file. Added depth for a few missing values from 2016.
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/beaulieu_jake_epa_gov/Documents/gitRepository/SuRGE/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30E28EBA-695B-4B28-8321-9B2E01519D99}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5BB1541-24BC-4185-B360-2E8261798A7C}"/>
   <bookViews>
-    <workbookView xWindow="4488" yWindow="5112" windowWidth="40200" windowHeight="12516" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="18576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1312,6 +1312,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -2637,6 +2641,9 @@
       <c r="L10" t="s">
         <v>198</v>
       </c>
+      <c r="W10">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="11" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
@@ -4357,8 +4364,45 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4833,45 +4877,8 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4883,9 +4890,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4914,15 +4927,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fixed transcription errors in chemistry files. Imputed missing sonde data for site 11 in lake 70-riverine. Committing to master. Need to make changes in data_paper branch.
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/beaulieu_jake_epa_gov/Documents/gitRepository/SuRGE/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5BB1541-24BC-4185-B360-2E8261798A7C}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9BF9627-203C-4B26-843D-3E1FFB28C752}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="18576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,6 +35,186 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={45E59198-3FB6-434C-8FE4-0BEEB2565B87}</author>
+    <author>tc={145F969C-530B-4108-A5CD-04ED45E333BC}</author>
+    <author>tc={92C78109-BF18-41E4-B726-55620B95DDD5}</author>
+    <author>tc={39DCBD55-9790-487A-871D-F4735B7FE117}</author>
+    <author>tc={AF67C030-F32B-4DDE-9A1E-4FD1FAA3ABA0}</author>
+    <author>tc={23C01AA2-E974-44B2-A95B-AD2FEDE3F9D6}</author>
+    <author>tc={91031D82-219F-4C21-B7B5-9781BB1775F4}</author>
+    <author>tc={499B4D21-4816-418F-ADF4-DD64214ED74A}</author>
+    <author>tc={9F30236F-D8E3-4591-8F90-FB9C60DDF127}</author>
+    <author>tc={53FC60D9-52C7-4650-AA7B-D4A2B7F38235}</author>
+    <author>tc={DCD82851-20C9-4724-96A8-41A2647819E9}</author>
+    <author>tc={5B0B7E90-0047-4BDA-B5F5-6687ACF3C8EA}</author>
+    <author>tc={51132BA8-C28C-4BF8-B4DA-7A2638662E1B}</author>
+    <author>tc={DCA8B116-1B1D-40C5-B727-B9302988877F}</author>
+    <author>tc={FA02D264-6E57-4D02-9BDF-B4FF921E3AAD}</author>
+    <author>tc={558F31AF-1B65-409F-B4AE-6042DA1D4BBC}</author>
+    <author>tc={22D4AC18-D728-4F52-A192-6B1F6ED6F61D}</author>
+    <author>tc={AD704169-B691-4DBC-AA56-EE79683AE7DE}</author>
+    <author>tc={10936FD2-6AB7-4772-91D6-FA37E720AA4F}</author>
+  </authors>
+  <commentList>
+    <comment ref="Y10" authorId="0" shapeId="0" xr:uid="{45E59198-3FB6-434C-8FE4-0BEEB2565B87}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="Z10" authorId="1" shapeId="0" xr:uid="{145F969C-530B-4108-A5CD-04ED45E333BC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AA10" authorId="2" shapeId="0" xr:uid="{92C78109-BF18-41E4-B726-55620B95DDD5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AB10" authorId="3" shapeId="0" xr:uid="{39DCBD55-9790-487A-871D-F4735B7FE117}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AC10" authorId="4" shapeId="0" xr:uid="{AF67C030-F32B-4DDE-9A1E-4FD1FAA3ABA0}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AD10" authorId="5" shapeId="0" xr:uid="{23C01AA2-E974-44B2-A95B-AD2FEDE3F9D6}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AQ10" authorId="6" shapeId="0" xr:uid="{91031D82-219F-4C21-B7B5-9781BB1775F4}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AR10" authorId="7" shapeId="0" xr:uid="{499B4D21-4816-418F-ADF4-DD64214ED74A}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AS10" authorId="8" shapeId="0" xr:uid="{9F30236F-D8E3-4591-8F90-FB9C60DDF127}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AT10" authorId="9" shapeId="0" xr:uid="{53FC60D9-52C7-4650-AA7B-D4A2B7F38235}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AU10" authorId="10" shapeId="0" xr:uid="{DCD82851-20C9-4724-96A8-41A2647819E9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AV10" authorId="11" shapeId="0" xr:uid="{5B0B7E90-0047-4BDA-B5F5-6687ACF3C8EA}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AW10" authorId="12" shapeId="0" xr:uid="{51132BA8-C28C-4BF8-B4DA-7A2638662E1B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AR14" authorId="13" shapeId="0" xr:uid="{DCA8B116-1B1D-40C5-B727-B9302988877F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AS14" authorId="14" shapeId="0" xr:uid="{FA02D264-6E57-4D02-9BDF-B4FF921E3AAD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AT14" authorId="15" shapeId="0" xr:uid="{558F31AF-1B65-409F-B4AE-6042DA1D4BBC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AU14" authorId="16" shapeId="0" xr:uid="{22D4AC18-D728-4F52-A192-6B1F6ED6F61D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AV14" authorId="17" shapeId="0" xr:uid="{AD704169-B691-4DBC-AA56-EE79683AE7DE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AW14" authorId="18" shapeId="0" xr:uid="{10936FD2-6AB7-4772-91D6-FA37E720AA4F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="199">
   <si>
@@ -646,7 +826,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -786,6 +966,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="39">
@@ -1313,7 +1499,9 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Beaulieu, Jake" id="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" userId="S::Beaulieu.Jake@epa.gov::f0420c56-494d-43d8-8142-91ff9a3846e6" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1611,8 +1799,70 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="Y10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{45E59198-3FB6-434C-8FE4-0BEEB2565B87}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="Z10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{145F969C-530B-4108-A5CD-04ED45E333BC}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AA10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{92C78109-BF18-41E4-B726-55620B95DDD5}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AB10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{39DCBD55-9790-487A-871D-F4735B7FE117}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AC10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{AF67C030-F32B-4DDE-9A1E-4FD1FAA3ABA0}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AD10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{23C01AA2-E974-44B2-A95B-AD2FEDE3F9D6}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AQ10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{91031D82-219F-4C21-B7B5-9781BB1775F4}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AR10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{499B4D21-4816-418F-ADF4-DD64214ED74A}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AS10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{9F30236F-D8E3-4591-8F90-FB9C60DDF127}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AT10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{53FC60D9-52C7-4650-AA7B-D4A2B7F38235}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AU10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{DCD82851-20C9-4724-96A8-41A2647819E9}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AV10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{5B0B7E90-0047-4BDA-B5F5-6687ACF3C8EA}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AW10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{51132BA8-C28C-4BF8-B4DA-7A2638662E1B}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AR14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{DCA8B116-1B1D-40C5-B727-B9302988877F}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AS14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{FA02D264-6E57-4D02-9BDF-B4FF921E3AAD}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AT14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{558F31AF-1B65-409F-B4AE-6042DA1D4BBC}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AU14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{22D4AC18-D728-4F52-A192-6B1F6ED6F61D}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AV14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{AD704169-B691-4DBC-AA56-EE79683AE7DE}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AW14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{10936FD2-6AB7-4772-91D6-FA37E720AA4F}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BP17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2644,6 +2894,48 @@
       <c r="W10">
         <v>5.8</v>
       </c>
+      <c r="X10">
+        <v>0.1</v>
+      </c>
+      <c r="Y10">
+        <v>23.4</v>
+      </c>
+      <c r="Z10">
+        <v>8.1</v>
+      </c>
+      <c r="AA10">
+        <v>870</v>
+      </c>
+      <c r="AB10">
+        <v>8.5</v>
+      </c>
+      <c r="AC10">
+        <v>0.8</v>
+      </c>
+      <c r="AD10">
+        <v>9</v>
+      </c>
+      <c r="AQ10">
+        <v>5</v>
+      </c>
+      <c r="AR10">
+        <v>22.4</v>
+      </c>
+      <c r="AS10">
+        <v>8</v>
+      </c>
+      <c r="AT10">
+        <v>870</v>
+      </c>
+      <c r="AU10">
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="AV10">
+        <v>1.45</v>
+      </c>
+      <c r="AW10">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
@@ -2977,6 +3269,27 @@
         <v>1.4</v>
       </c>
       <c r="AD14">
+        <v>14.4</v>
+      </c>
+      <c r="AQ14">
+        <v>1</v>
+      </c>
+      <c r="AR14">
+        <v>23</v>
+      </c>
+      <c r="AS14">
+        <v>8.6</v>
+      </c>
+      <c r="AT14">
+        <v>865</v>
+      </c>
+      <c r="AU14">
+        <v>8.4</v>
+      </c>
+      <c r="AV14">
+        <v>1.4</v>
+      </c>
+      <c r="AW14">
         <v>14.4</v>
       </c>
     </row>
@@ -3259,6 +3572,7 @@
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4355,15 +4669,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
@@ -4405,7 +4710,21 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF5FC5DD832BE4DBA6B24560DD3ADC0" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d40b3e6283001fb57e5088f84fb23d5e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="8b03727f-4454-4722-b3e6-018d8dcaf2fd" xmlns:ns6="ed970698-2d60-4bab-a048-d9be527522d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aadbb8160917885bdc8cfb32badaafe9" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4876,20 +5195,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4903,7 +5209,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F85A6490-A4FD-48A0-8CAA-E2B88EB380BB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4924,12 +5246,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Integrating water chemistry fixes that were first implemented in master branch.
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/surgeData70Riverine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/beaulieu_jake_epa_gov/Documents/gitRepository/SuRGE/SuRGE_Sharepoint/data/CIN/CH4_070_francis_case_riverine/dataSheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5BB1541-24BC-4185-B360-2E8261798A7C}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{2FA17500-E920-4072-996D-0191A222BF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9BF9627-203C-4B26-843D-3E1FFB28C752}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="18576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,6 +35,186 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={45E59198-3FB6-434C-8FE4-0BEEB2565B87}</author>
+    <author>tc={145F969C-530B-4108-A5CD-04ED45E333BC}</author>
+    <author>tc={92C78109-BF18-41E4-B726-55620B95DDD5}</author>
+    <author>tc={39DCBD55-9790-487A-871D-F4735B7FE117}</author>
+    <author>tc={AF67C030-F32B-4DDE-9A1E-4FD1FAA3ABA0}</author>
+    <author>tc={23C01AA2-E974-44B2-A95B-AD2FEDE3F9D6}</author>
+    <author>tc={91031D82-219F-4C21-B7B5-9781BB1775F4}</author>
+    <author>tc={499B4D21-4816-418F-ADF4-DD64214ED74A}</author>
+    <author>tc={9F30236F-D8E3-4591-8F90-FB9C60DDF127}</author>
+    <author>tc={53FC60D9-52C7-4650-AA7B-D4A2B7F38235}</author>
+    <author>tc={DCD82851-20C9-4724-96A8-41A2647819E9}</author>
+    <author>tc={5B0B7E90-0047-4BDA-B5F5-6687ACF3C8EA}</author>
+    <author>tc={51132BA8-C28C-4BF8-B4DA-7A2638662E1B}</author>
+    <author>tc={DCA8B116-1B1D-40C5-B727-B9302988877F}</author>
+    <author>tc={FA02D264-6E57-4D02-9BDF-B4FF921E3AAD}</author>
+    <author>tc={558F31AF-1B65-409F-B4AE-6042DA1D4BBC}</author>
+    <author>tc={22D4AC18-D728-4F52-A192-6B1F6ED6F61D}</author>
+    <author>tc={AD704169-B691-4DBC-AA56-EE79683AE7DE}</author>
+    <author>tc={10936FD2-6AB7-4772-91D6-FA37E720AA4F}</author>
+  </authors>
+  <commentList>
+    <comment ref="Y10" authorId="0" shapeId="0" xr:uid="{45E59198-3FB6-434C-8FE4-0BEEB2565B87}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="Z10" authorId="1" shapeId="0" xr:uid="{145F969C-530B-4108-A5CD-04ED45E333BC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AA10" authorId="2" shapeId="0" xr:uid="{92C78109-BF18-41E4-B726-55620B95DDD5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AB10" authorId="3" shapeId="0" xr:uid="{39DCBD55-9790-487A-871D-F4735B7FE117}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AC10" authorId="4" shapeId="0" xr:uid="{AF67C030-F32B-4DDE-9A1E-4FD1FAA3ABA0}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AD10" authorId="5" shapeId="0" xr:uid="{23C01AA2-E974-44B2-A95B-AD2FEDE3F9D6}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AQ10" authorId="6" shapeId="0" xr:uid="{91031D82-219F-4C21-B7B5-9781BB1775F4}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AR10" authorId="7" shapeId="0" xr:uid="{499B4D21-4816-418F-ADF4-DD64214ED74A}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AS10" authorId="8" shapeId="0" xr:uid="{9F30236F-D8E3-4591-8F90-FB9C60DDF127}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AT10" authorId="9" shapeId="0" xr:uid="{53FC60D9-52C7-4650-AA7B-D4A2B7F38235}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AU10" authorId="10" shapeId="0" xr:uid="{DCD82851-20C9-4724-96A8-41A2647819E9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AV10" authorId="11" shapeId="0" xr:uid="{5B0B7E90-0047-4BDA-B5F5-6687ACF3C8EA}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AW10" authorId="12" shapeId="0" xr:uid="{51132BA8-C28C-4BF8-B4DA-7A2638662E1B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Not recorded in field. Imputed from nearby sites/</t>
+      </text>
+    </comment>
+    <comment ref="AR14" authorId="13" shapeId="0" xr:uid="{DCA8B116-1B1D-40C5-B727-B9302988877F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AS14" authorId="14" shapeId="0" xr:uid="{FA02D264-6E57-4D02-9BDF-B4FF921E3AAD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AT14" authorId="15" shapeId="0" xr:uid="{558F31AF-1B65-409F-B4AE-6042DA1D4BBC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AU14" authorId="16" shapeId="0" xr:uid="{22D4AC18-D728-4F52-A192-6B1F6ED6F61D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AV14" authorId="17" shapeId="0" xr:uid="{AD704169-B691-4DBC-AA56-EE79683AE7DE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+    <comment ref="AW14" authorId="18" shapeId="0" xr:uid="{10936FD2-6AB7-4772-91D6-FA37E720AA4F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assuming equivalency with shallow measurements.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="199">
   <si>
@@ -646,7 +826,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -786,6 +966,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="39">
@@ -1313,7 +1499,9 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Beaulieu, Jake" id="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" userId="S::Beaulieu.Jake@epa.gov::f0420c56-494d-43d8-8142-91ff9a3846e6" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1611,8 +1799,70 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="Y10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{45E59198-3FB6-434C-8FE4-0BEEB2565B87}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="Z10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{145F969C-530B-4108-A5CD-04ED45E333BC}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AA10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{92C78109-BF18-41E4-B726-55620B95DDD5}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AB10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{39DCBD55-9790-487A-871D-F4735B7FE117}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AC10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{AF67C030-F32B-4DDE-9A1E-4FD1FAA3ABA0}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AD10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{23C01AA2-E974-44B2-A95B-AD2FEDE3F9D6}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AQ10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{91031D82-219F-4C21-B7B5-9781BB1775F4}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AR10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{499B4D21-4816-418F-ADF4-DD64214ED74A}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AS10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{9F30236F-D8E3-4591-8F90-FB9C60DDF127}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AT10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{53FC60D9-52C7-4650-AA7B-D4A2B7F38235}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AU10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{DCD82851-20C9-4724-96A8-41A2647819E9}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AV10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{5B0B7E90-0047-4BDA-B5F5-6687ACF3C8EA}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AW10" dT="2025-08-13T13:10:13.99" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{51132BA8-C28C-4BF8-B4DA-7A2638662E1B}">
+    <text>Not recorded in field. Imputed from nearby sites/</text>
+  </threadedComment>
+  <threadedComment ref="AR14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{DCA8B116-1B1D-40C5-B727-B9302988877F}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AS14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{FA02D264-6E57-4D02-9BDF-B4FF921E3AAD}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AT14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{558F31AF-1B65-409F-B4AE-6042DA1D4BBC}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AU14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{22D4AC18-D728-4F52-A192-6B1F6ED6F61D}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AV14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{AD704169-B691-4DBC-AA56-EE79683AE7DE}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+  <threadedComment ref="AW14" dT="2025-08-13T13:14:29.69" personId="{95D37A7A-073E-47AC-9ABD-C1E3B91E2E11}" id="{10936FD2-6AB7-4772-91D6-FA37E720AA4F}">
+    <text>Assuming equivalency with shallow measurements.</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BP17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2644,6 +2894,48 @@
       <c r="W10">
         <v>5.8</v>
       </c>
+      <c r="X10">
+        <v>0.1</v>
+      </c>
+      <c r="Y10">
+        <v>23.4</v>
+      </c>
+      <c r="Z10">
+        <v>8.1</v>
+      </c>
+      <c r="AA10">
+        <v>870</v>
+      </c>
+      <c r="AB10">
+        <v>8.5</v>
+      </c>
+      <c r="AC10">
+        <v>0.8</v>
+      </c>
+      <c r="AD10">
+        <v>9</v>
+      </c>
+      <c r="AQ10">
+        <v>5</v>
+      </c>
+      <c r="AR10">
+        <v>22.4</v>
+      </c>
+      <c r="AS10">
+        <v>8</v>
+      </c>
+      <c r="AT10">
+        <v>870</v>
+      </c>
+      <c r="AU10">
+        <v>8.4499999999999993</v>
+      </c>
+      <c r="AV10">
+        <v>1.45</v>
+      </c>
+      <c r="AW10">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
@@ -2977,6 +3269,27 @@
         <v>1.4</v>
       </c>
       <c r="AD14">
+        <v>14.4</v>
+      </c>
+      <c r="AQ14">
+        <v>1</v>
+      </c>
+      <c r="AR14">
+        <v>23</v>
+      </c>
+      <c r="AS14">
+        <v>8.6</v>
+      </c>
+      <c r="AT14">
+        <v>865</v>
+      </c>
+      <c r="AU14">
+        <v>8.4</v>
+      </c>
+      <c r="AV14">
+        <v>1.4</v>
+      </c>
+      <c r="AW14">
         <v>14.4</v>
       </c>
     </row>
@@ -3259,6 +3572,7 @@
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4355,15 +4669,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
@@ -4405,7 +4710,21 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF5FC5DD832BE4DBA6B24560DD3ADC0" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d40b3e6283001fb57e5088f84fb23d5e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="8b03727f-4454-4722-b3e6-018d8dcaf2fd" xmlns:ns6="ed970698-2d60-4bab-a048-d9be527522d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aadbb8160917885bdc8cfb32badaafe9" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4876,20 +5195,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4903,7 +5209,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F85A6490-A4FD-48A0-8CAA-E2B88EB380BB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4924,12 +5246,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>